<commit_message>
some more sample leads add to excel
</commit_message>
<xml_diff>
--- a/data/leads_crm.xlsx
+++ b/data/leads_crm.xlsx
@@ -8,19 +8,30 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AI Voice Sales Agent\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7EA437A-F794-4809-A9EE-32D3A85F4D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CD22EC5-EFE1-4C2B-A010-8E14F9FD1039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Leads" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="81">
   <si>
     <t>Lead ID</t>
   </si>
@@ -188,13 +199,88 @@
   </si>
   <si>
     <t>karan@malhotraauto.com</t>
+  </si>
+  <si>
+    <t>L006</t>
+  </si>
+  <si>
+    <t>L007</t>
+  </si>
+  <si>
+    <t>L008</t>
+  </si>
+  <si>
+    <t>L009</t>
+  </si>
+  <si>
+    <t>L010</t>
+  </si>
+  <si>
+    <t>Vishesh Unadkat</t>
+  </si>
+  <si>
+    <t>Nirmit Patel</t>
+  </si>
+  <si>
+    <t>Priyank Viradiya</t>
+  </si>
+  <si>
+    <t>Yug Sakariya</t>
+  </si>
+  <si>
+    <t>Hari Solanki</t>
+  </si>
+  <si>
+    <t>"+91-9876512345"</t>
+  </si>
+  <si>
+    <t>"+91-9823012345"</t>
+  </si>
+  <si>
+    <t>"+91-9811123456"</t>
+  </si>
+  <si>
+    <t>"+91-9845012345"</t>
+  </si>
+  <si>
+    <t>"+91-9834512345"</t>
+  </si>
+  <si>
+    <t>Unadkat Technologies</t>
+  </si>
+  <si>
+    <t>Patel Agro Solutions</t>
+  </si>
+  <si>
+    <t>Shah Digital Marketing</t>
+  </si>
+  <si>
+    <t>Joshi Electronics</t>
+  </si>
+  <si>
+    <t>Desai Foods Pvt Ltd</t>
+  </si>
+  <si>
+    <t>vishesh@unadkattech.com</t>
+  </si>
+  <si>
+    <t>nirmit@patelagro.com</t>
+  </si>
+  <si>
+    <t>priyank@shahdigital.in</t>
+  </si>
+  <si>
+    <t>yug@joshielectronics.com</t>
+  </si>
+  <si>
+    <t>hari@desaifoods.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -211,6 +297,14 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -235,10 +329,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -246,8 +341,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -548,11 +650,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="3" width="16" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
@@ -779,7 +882,114 @@
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
     </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" t="s">
+        <v>68</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E7" r:id="rId1" xr:uid="{77383F83-423C-4025-BF29-9971C6C150D3}"/>
+    <hyperlink ref="E8" r:id="rId2" xr:uid="{D461AA06-19F0-4A30-9198-35D089F33A91}"/>
+    <hyperlink ref="E9" r:id="rId3" xr:uid="{62B442AB-2158-4967-B479-E0224ACAF411}"/>
+    <hyperlink ref="E10" r:id="rId4" xr:uid="{11F96918-69D9-48E9-A678-5BEFD3D86AE0}"/>
+    <hyperlink ref="E11" r:id="rId5" xr:uid="{BF363E5D-B881-4B62-B2EE-57DB6C5D6DC0}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>